<commit_message>
Chatbot Workflow completed with testcases
</commit_message>
<xml_diff>
--- a/test_data/Query.xlsx
+++ b/test_data/Query.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
+          <t>&lt;आई. डी. १७२३&gt;, २०२६ पर शाखा ००१ क कुल सदस्यक गिनती ३,५०४ छल।</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
+          <t>Thinking …</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
+          <t>Thinking …</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
+          <t>Thinking …</t>
         </is>
       </c>
     </row>
@@ -484,187 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>As of Feb 14, How many total employees does Branch 001 have, and what is the gender breakdown?</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>On the last day of February, what was the total number of employees across all branches?</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>What was the saving deposit of Branch 004 on January 15, 2026?</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>deposit counts on feb 10 2026</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>How many deposit counts did Branch 005 have on February 10, 2026?</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>What is the total number of borrowers in Branch 001 as of April 30 2024?</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Which branch has the highest number of members as of February 28, 2026?</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Which branch had more dropouts in 2022?</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Which branch has the fewest members as of February 28, 2026?</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Compare the borrower-to-member ratio across all branches as of February 28, 2026.</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>How did the number of borrowers in branch 005 changed from first day of January to February last</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>What percentage of Branch 002's total members were male on February 28, 2026? (Round to 2 decimal places)</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>How did Branch 001's saving deposit change from January 1 to January 15 to January 31?</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Track Branch 002's member count at four points: Jan 1, Jan 15, Feb 1, Feb 28</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Compare Branch 002's saving deposit trajectory: Jan 1 → Jan 20 → Feb 10 → Feb 28.</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Hello! I am WiseAI. How can I help you today?</t>
+          <t>Thinking …</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Changed File Structure and markers
</commit_message>
<xml_diff>
--- a/test_data/Query.xlsx
+++ b/test_data/Query.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,60 +431,288 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>What was the total member count for Branch 001 on January 15?</t>
+          <t>What is the ideal soil pH for tomato cultivation?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>&lt;आई. डी. १७२३&gt;, २०२६ पर शाखा ००१ क कुल सदस्यक गिनती ३,५०४ छल।</t>
+          <t>टमाटर खेतीका लागि आदर्श माटोको pH ६ र ७ को बिचमा हुन्छ।</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>What was branch 001's saving deposit on Jan 1 last year?</t>
+          <t>Which temperature range is best for tomato cultivation?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Thinking …</t>
+          <t>टमाटर खेतीका लागि उपयुक्त तापमान दायरा २० डिग्री सेल्सियस देखि २५ डिग्री सेल्सियस छ, तापमान १६ डिग्री सेल्सियस भन्दा कम र २७ डिग्री सेल्सियस भन्दा माथि अनुपयुक्त छ।</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>What is the membership growth trend for Branch 001 from Feb 14 to Feb 28</t>
+          <t>How much tomato seed is needed for one ropani?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Thinking …</t>
+          <t>एउटा रोपनीमा टमाटर खेती गर्न लगभग १० ग्राम बिउ चाहिन्छ।</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>What was the total Saving Deposit amount for Branch 001 on the first day of January?</t>
+          <t>At what leaf stage should tomato seedlings be transplanted?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Thinking …</t>
+          <t>टमाटरका बिरुवाहरू ४-५ पातको चरणमा हुँदा प्रत्यारोपण गर्नुपर्छ, जुन लगभग २५ दिन पुरानो हो।</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>What is the non collateral loan of Branch 001 on Jan 1 2021?</t>
+          <t>What is the recommended spacing for tomato plants?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Thinking …</t>
+          <t>टमाटरका बिरुवाका लागि सिफारिस गरिएको दुरी बिरुवाहरू बिच ६० सेन्टिमिटर र पङ्क्तिहरू बिच ६० सेन्टिमिटर छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Which irrigation method is preferred for tomato under plastic house?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>प्लास्टिक घरहरूअन्तर्गत, टमेटाका लागि सिँचाइ विशेष गरी ड्रिप इरिगेसनद्वारा गरिन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>How often should tomato be irrigated?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>माटोको अवस्थाका आधारमा प्रत्येक ५ देखि ७ दिनमा टमाटर सिँचाइ गर्नुपर्छ, यदि प्लास्टिकको घरमुनि उब्जाएको भए पनि वर्षाको मौसममा पनि नियमित सिँचाईलाई प्राथमिकता दिइन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>What happens when temperature rises above 35°C in tomato?</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>जब तापक्रम ३५ डिग्री सेल्सियसभन्दा माथि बढ्छ, परागको दाना सुकेको हुन्छ, जसले गर्दा खराब फलको सेट हुन्छ; फलको सेट भए पनि, फलको आकार विकृत हुन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Which disease causes wrinkled and curled tomato leaves?</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>लिफ कर्ल भाइरसले टमाटरका पातहरू चुचुरो वा पकर भएको देखिन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>What is the best temperature for tomato fruit setting?</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>टमाटर फलको सेटिङका लागि उत्तम तापमान २५ डिग्री सेल्सियसदेखि २८ डिग्री सेल्सियस हुन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Which fungicide is recommended for late blight management?</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>लेट ब्लाइट (फ्रुट रोट) व्यवस्थापनका लागि सिफारिस गरिएका ढुसीनाशकहरू डिथेन एम-४५, सेक्टिन (फेमितोडिन), वा रियलवेट/डायमंड (डाइमेथोमोर्फ) हुन्।</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Which pest can be controlled using yellow sticky traps?</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>सेतो झिँगाहरू पहेँलो चिपचिपा जालहरू प्रयोग गरेर नियन्त्रण गर्न सकिन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Which trap crop is used against tomato fruit borer?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>गाँजा टमाटरको फल छेड्ने विरुद्धमा जाल बालीको रूपमा प्रयोग गरिन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>What is the major symptom of root-knot nematode?</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>जरा-गाँठ नेमाटोडको प्रमुख लक्षण टमाटरको जरामा गलको गठन हो, जसले उचित वृद्धि र पोषक तत्वहरूको अवशोषणलाई रोक्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>What should be the age of tomato seedlings during transplanting?</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>टमाटरका बिरुवाहरू ४-५ पातको चरणमा हुँदा प्रत्यारोपण गर्नुपर्छ, जुन लगभग २५ दिन पुरानो हो।</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Which disease causes sudden wilting with white bacterial ooze from the stem?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ब्याक्टेरियल विल्टले स्टेमबाट सेतो, चिपचिपा ब्याक्टेरियल ओज निस्कँदा अचानक सुकेको हुन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Which nutrient deficiency increases fruit cracking in tomato?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>बोरोनको कमीले टमाटरमा फलको क्र्याकिङ बढाउँछ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>What is the main purpose of tomato grafting?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>टमाटर कलम बनाउने मुख्य उद्देश्य रोग प्रतिरोधी जरा प्रयोग गरेर ब्याक्टेरियल विल्ट र रुट-नट नेमाटोडको घटना घटाउनु हो, जसले उत्पादन पनि २२ देखि ३८ प्रतिशतले बढाउँछ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>How much yield can tall tomato varieties produce per plant under good management?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>राम्रो व्यवस्थापन अन्तर्गत, अग्लो टमाटरका प्रजातिहरूले प्रति बिरुवा १०-१५ किलोग्राम उत्पादन गर्न सक्छन्।</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>What is the recommended temperature range for tomato seed germination?</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>टमाटरको बिउ अङ्कुरणका लागि, सिफारिस गरिएको तापमान दायरा १८ डिग्री सेल्सियस र २६ डिग्री सेल्सियसको बिचमा हुन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>how much space is required for tomato plantation?</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>एउटा रोपनी जमिनमा टमाटर खेती गर्न ६ वर्ग मिटरको नर्सरी क्षेत्र चाहिन्छ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>what does tomato grafting do?</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>टमेटाको कलमले रोग प्रतिरोधी जरा प्रयोग गरेर ब्याक्टेरियल विल्ट र रुट-नट नेमाटोडको घटना घटाउँछ, जसले उत्पादन पनि २२ देखि ३८ प्रतिशतले बढाउँछ।</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Can I use tomato seedlings of 5 days for transplanting?</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>म यसको जवाफ दिन सक्दिनँ किनभने यो प्रदान गरिएको सन्दर्भमा समावेश छैन।</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Calculate the standard tomato seed requirement (in grams) needed to cultivate an area of one ropani.</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>एक रोपानी जमिनमा खेती गर्न लगभग १० ग्राम टमाटरको बिउ चाहिन्छ।</t>
         </is>
       </c>
     </row>

</xml_diff>